<commit_message>
Accounting-start slicer, sign-up from the login screen, operations log files, default accounts in the delivered workbook
- Engine override lets the dashboard/insights/ledger/BI pick the year arrears are counted from without touching the setting or the workbook
- Login screen offers «حساب جديد» (staff account written to the users sheet); first-run/recovery screens stay as fallbacks
- Operations log: every change, login, logout and refused login buffered in the browser and appended to monthly CSV files under backups/logs when the folder is enabled; settings card with CSV download
- Tests: log suite, slicer override, e2e 18; guides updated

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199m3xvAaJoQxvDRKzxjRoJ
</commit_message>
<xml_diff>
--- a/Egary/Egary.xlsx
+++ b/Egary/Egary.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8677" uniqueCount="1294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8683" uniqueCount="1299">
   <si>
     <t>إيجاري</t>
   </si>
@@ -1674,7 +1674,7 @@
     <t>01/04/2026</t>
   </si>
   <si>
-    <t>تنتهي قريبًا</t>
+    <t>تنتهي خلال 90 يومًا</t>
   </si>
   <si>
     <t>ending</t>
@@ -3792,6 +3792,21 @@
     <t>أوراق السنوات الموجودة (تُضاف تلقائيًا)</t>
   </si>
   <si>
+    <t>أعلى أرقام الأكواد الصادرة</t>
+  </si>
+  <si>
+    <t>{"P":3,"C":64,"T":86,"INV-2026":509}</t>
+  </si>
+  <si>
+    <t>لا تُعدَّل: تضمن ألا يُعاد استخدام كود محذوف</t>
+  </si>
+  <si>
+    <t>بداية المحاسبة (تلقائي/يدوي)</t>
+  </si>
+  <si>
+    <t>auto = تبدأ من أقدم ورقة سنة · manual = كما ضبطها المدير</t>
+  </si>
+  <si>
     <t>بادئة رقم الفاتورة</t>
   </si>
   <si>
@@ -3840,7 +3855,7 @@
     <t>آخر كتابة من الموقع</t>
   </si>
   <si>
-    <t>2026-10-10 10:52:13</t>
+    <t>2026-10-10 12:59:59</t>
   </si>
   <si>
     <t>إصدار البنية</t>
@@ -3882,7 +3897,7 @@
     <t>مدير</t>
   </si>
   <si>
-    <t>pbkdf2$120000$b0516fecda139ffd23f828131551415c$52e12d9c59ccf4e48ddba28948deb330f3ffecfcfdf979d4942dc5d6107940c5</t>
+    <t>pbkdf2$120000$2a399ba5667533b4f0c3539ea2dda9bc$c81d26d23246b2f03b92df85e7472919122554f3f09d819ef7b916caccf10cd3</t>
   </si>
   <si>
     <t>office</t>
@@ -3894,7 +3909,7 @@
     <t>موظف</t>
   </si>
   <si>
-    <t>pbkdf2$120000$b58a51da6139631be1f358a8d09f194d$5961a914482fc5a83e7294521c86e7506bb15ecf7ff304dd71ff2d06231df0c6</t>
+    <t>pbkdf2$120000$6e87cd2bc9f71469b0d2391c3c7b7019$40355bed31efb5e38d21aa3157e7a6f6821ef8a864666be2d9095e67f9bdba04</t>
   </si>
   <si>
     <t>zaer</t>
@@ -3906,7 +3921,7 @@
     <t>مشاهدة فقط</t>
   </si>
   <si>
-    <t>pbkdf2$120000$d4eafbbdc30de3c498a71b5655775c2e$38146298018fbec477acf08007af0b57233f11ac8d0c4e6b822514c9afc4debe</t>
+    <t>pbkdf2$120000$f7b621f0224fe71430628d668c922100$140188b3ee26c8c0e4f17ec926e93cc6fc18e463410f011aef10fe030acb4480</t>
   </si>
 </sst>
 </file>
@@ -11032,7 +11047,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -11144,18 +11159,18 @@
         <v>1258</v>
       </c>
       <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
         <v>1259</v>
-      </c>
-      <c r="C10" t="s">
-        <v>1260</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>1260</v>
+      </c>
+      <c r="B11" t="s">
         <v>1261</v>
-      </c>
-      <c r="B11" t="s">
-        <v>35</v>
       </c>
       <c r="C11" t="s">
         <v>1262</v>
@@ -11165,48 +11180,70 @@
       <c r="A12" t="s">
         <v>1263</v>
       </c>
-      <c r="B12">
-        <v>0.5</v>
+      <c r="B12" t="s">
+        <v>1264</v>
       </c>
       <c r="C12" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1265</v>
-      </c>
-      <c r="B13">
-        <v>50</v>
+        <v>1266</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B14" t="s">
         <v>1268</v>
+      </c>
+      <c r="B14">
+        <v>0.5</v>
       </c>
       <c r="C14" t="s">
         <v>1269</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>1270</v>
+      </c>
+      <c r="B15">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>1270</v>
+        <v>1272</v>
       </c>
       <c r="B16" t="s">
-        <v>1271</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>1272</v>
-      </c>
-      <c r="B17">
+        <v>1273</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1275</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B19">
         <v>2</v>
       </c>
     </row>
@@ -11230,22 +11267,22 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>1273</v>
+        <v>1278</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1274</v>
+        <v>1279</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1275</v>
+        <v>1280</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>1276</v>
+        <v>1281</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>565</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>1277</v>
+        <v>1282</v>
       </c>
     </row>
   </sheetData>
@@ -11270,7 +11307,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>1278</v>
+        <v>1283</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>4</v>
@@ -11279,30 +11316,30 @@
         <v>526</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>1279</v>
+        <v>1284</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>1280</v>
+        <v>1285</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>518</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>1281</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1282</v>
+        <v>1287</v>
       </c>
       <c r="B2" t="s">
-        <v>1283</v>
+        <v>1288</v>
       </c>
       <c r="C2" t="s">
-        <v>1284</v>
+        <v>1289</v>
       </c>
       <c r="D2" s="32" t="s">
-        <v>1285</v>
+        <v>1290</v>
       </c>
       <c r="E2" t="s">
         <v>687</v>
@@ -11316,16 +11353,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1286</v>
+        <v>1291</v>
       </c>
       <c r="B3" t="s">
-        <v>1287</v>
+        <v>1292</v>
       </c>
       <c r="C3" t="s">
-        <v>1288</v>
+        <v>1293</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>1289</v>
+        <v>1294</v>
       </c>
       <c r="E3" t="s">
         <v>687</v>
@@ -11339,16 +11376,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1290</v>
+        <v>1295</v>
       </c>
       <c r="B4" t="s">
-        <v>1291</v>
+        <v>1296</v>
       </c>
       <c r="C4" t="s">
-        <v>1292</v>
+        <v>1297</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>1293</v>
+        <v>1298</v>
       </c>
       <c r="E4" t="s">
         <v>687</v>

</xml_diff>